<commit_message>
Refresh DiDi transparent sheet after Mexico $30 premium fare (#288)
</commit_message>
<xml_diff>
--- a/finance/_refresh_didi.xlsx
+++ b/finance/_refresh_didi.xlsx
@@ -3579,7 +3579,7 @@
         <v>3.35</v>
       </c>
       <c r="E8" s="27" t="n">
-        <v>15.07</v>
+        <v>30</v>
       </c>
       <c r="F8" s="34" t="inlineStr">
         <is>
@@ -3588,7 +3588,7 @@
       </c>
       <c r="G8" s="34" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>med</t>
         </is>
       </c>
       <c r="H8" s="20" t="n">
@@ -3753,7 +3753,7 @@
       </c>
       <c r="AY8" s="46" t="inlineStr">
         <is>
-          <t>https://ultracarga.com/ruta-punta-sam-isla-mujeres/</t>
+          <t>https://www.uber.com/mx/en/ride/uber-black/</t>
         </is>
       </c>
       <c r="AZ8" s="46" t="inlineStr">
@@ -3967,7 +3967,7 @@
         <v>5.27</v>
       </c>
       <c r="E10" s="27" t="n">
-        <v>15.07</v>
+        <v>30</v>
       </c>
       <c r="F10" s="34" t="inlineStr">
         <is>
@@ -3976,7 +3976,7 @@
       </c>
       <c r="G10" s="34" t="inlineStr">
         <is>
-          <t>med-low</t>
+          <t>med</t>
         </is>
       </c>
       <c r="H10" s="20" t="n">
@@ -4141,7 +4141,7 @@
       </c>
       <c r="AY10" s="46" t="inlineStr">
         <is>
-          <t>https://www.ultramarferry.com/es/tarifas</t>
+          <t>https://www.uber.com/mx/en/ride/uber-black/</t>
         </is>
       </c>
       <c r="AZ10" s="46" t="inlineStr">
@@ -4355,7 +4355,7 @@
         <v>9.529999999999999</v>
       </c>
       <c r="E12" s="27" t="n">
-        <v>16.63</v>
+        <v>30</v>
       </c>
       <c r="F12" s="34" t="inlineStr">
         <is>
@@ -4364,7 +4364,7 @@
       </c>
       <c r="G12" s="34" t="inlineStr">
         <is>
-          <t>med-low</t>
+          <t>med</t>
         </is>
       </c>
       <c r="H12" s="20" t="n">
@@ -4529,7 +4529,7 @@
       </c>
       <c r="AY12" s="46" t="inlineStr">
         <is>
-          <t>https://www.ultramarferry.com/en/fares</t>
+          <t>https://www.uber.com/mx/en/ride/uber-black/</t>
         </is>
       </c>
       <c r="AZ12" s="46" t="inlineStr">

</xml_diff>

<commit_message>
Cascade #292 Brazil/Egypt TAM into gen, scoped corridors, sheets
After merging #292 (bindings + model corridors + partner aggs):
- gen_deck_economics: count pending_seal_route_ids in country total
- Cascade Angra/Floripa PROV into corridors-didi + corridors-indrive
- Re-aggregate didi/indrive; regenerate three generated-deck-economics
- Refresh DiDi + inDrive + master transparent sheets (Drive uploaded in place)

Brazil floor $56.6M / 199 boats; DiDi 5-rung TAM; Egypt 4-rung width-template ladder.
</commit_message>
<xml_diff>
--- a/finance/_refresh_didi.xlsx
+++ b/finance/_refresh_didi.xlsx
@@ -53,8 +53,8 @@
     <definedName name="load_sel">'Assumptions'!$B$49</definedName>
     <definedName name="revleg_sel">'Assumptions'!$B$50</definedName>
     <definedName name="country_opex">'Country opex'!$A$4:$G$5</definedName>
-    <definedName name="som_floor_fleet">'Corridor economics'!$D$23</definedName>
-    <definedName name="som_floor_rev">'Corridor economics'!$E$23</definedName>
+    <definedName name="som_floor_fleet">'Corridor economics'!$D$26</definedName>
+    <definedName name="som_floor_rev">'Corridor economics'!$E$26</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -2381,7 +2381,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BA24"/>
+  <dimension ref="A1:BA27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3156,25 +3156,17 @@
       </c>
       <c r="C6" s="32" t="inlineStr">
         <is>
-          <t>Praça XV Terminal (central Rio) → Cocotá Terminal (Ilha do Governador)</t>
+          <t>Beira Mar Terminal (continent) → Miramar Terminal (Florianopolis island)</t>
         </is>
       </c>
       <c r="D6" s="33" t="n">
-        <v>6</v>
+        <v>4.79</v>
       </c>
       <c r="E6" s="27" t="n">
-        <v>28</v>
-      </c>
-      <c r="F6" s="34" t="inlineStr">
-        <is>
-          <t>T1/T2</t>
-        </is>
-      </c>
-      <c r="G6" s="34" t="inlineStr">
-        <is>
-          <t>med-low</t>
-        </is>
-      </c>
+        <v>20</v>
+      </c>
+      <c r="F6" s="34" t="n"/>
+      <c r="G6" s="34" t="n"/>
       <c r="H6" s="20" t="n">
         <v>1</v>
       </c>
@@ -3279,16 +3271,16 @@
         <v/>
       </c>
       <c r="AH6" s="33" t="n">
-        <v>278607</v>
+        <v>6100556</v>
       </c>
       <c r="AI6" s="34" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="AJ6" s="34" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>med-low</t>
         </is>
       </c>
       <c r="AK6" s="41" t="n">
@@ -3335,19 +3327,15 @@
         <f>IF(((T6*pax_cap*load_full*IF(ABS(MOD(ABS((L6*M6*revleg_full)),1)-0.5)&lt;1E-9,2*ROUND((L6*M6*revleg_full)/2,0),ROUND((L6*M6*revleg_full),0)))-(((battery/range_nm)*D6*IF(ABS(MOD(ABS((L6*M6*revleg_full)),1)-0.5)&lt;1E-9,2*ROUND((L6*M6*revleg_full)/2,0),ROUND((L6*M6*revleg_full),0))*VLOOKUP(B6,country_opex,3,FALSE))+W6+X6+Y6+Z6+AA6))&lt;=0,"",VLOOKUP(B6,country_opex,7,FALSE)/((T6*pax_cap*load_full*IF(ABS(MOD(ABS((L6*M6*revleg_full)),1)-0.5)&lt;1E-9,2*ROUND((L6*M6*revleg_full)/2,0),ROUND((L6*M6*revleg_full),0)))-(((battery/range_nm)*D6*IF(ABS(MOD(ABS((L6*M6*revleg_full)),1)-0.5)&lt;1E-9,2*ROUND((L6*M6*revleg_full)/2,0),ROUND((L6*M6*revleg_full),0))*VLOOKUP(B6,country_opex,3,FALSE))+W6+X6+Y6+Z6+AA6)))</f>
         <v/>
       </c>
-      <c r="AY6" s="46" t="inlineStr">
-        <is>
-          <t>https://barcasrio.com.br/linhas-horarios-e-tarifas/</t>
-        </is>
-      </c>
+      <c r="AY6" s="46" t="n"/>
       <c r="AZ6" s="46" t="inlineStr">
         <is>
-          <t>https://www2.agetransp.rj.gov.br/arquivos/operacao-servicos/relatorio-de-atividades/Relat%C3%B3rio%20Mensal%20de%20Atividades%20Janeiro%202024.pdf</t>
+          <t>https://www.sie.sc.gov.br/webdocs/sie/doc-tecnicos/aquaviario/ (EVTE Aquaviario RMF, Relatorio 3 - Componente Demanda; SIE-SC + BID)</t>
         </is>
       </c>
       <c r="BA6" s="34" t="inlineStr">
         <is>
-          <t>rn-369ef0eb69d9</t>
+          <t>rn-floripa-r4-PROV</t>
         </is>
       </c>
     </row>
@@ -3364,25 +3352,17 @@
       </c>
       <c r="C7" s="32" t="inlineStr">
         <is>
-          <t>Praça XV Terminal (central Rio) → Paquetá Island Terminal</t>
+          <t>Barreiros Terminal (Sao Jose / continent) → Miramar Terminal (Florianopolis island)</t>
         </is>
       </c>
       <c r="D7" s="33" t="n">
-        <v>9.199999999999999</v>
+        <v>4.99</v>
       </c>
       <c r="E7" s="27" t="n">
-        <v>28</v>
-      </c>
-      <c r="F7" s="34" t="inlineStr">
-        <is>
-          <t>T1/T2</t>
-        </is>
-      </c>
-      <c r="G7" s="34" t="inlineStr">
-        <is>
-          <t>med-low</t>
-        </is>
-      </c>
+        <v>20</v>
+      </c>
+      <c r="F7" s="34" t="n"/>
+      <c r="G7" s="34" t="n"/>
       <c r="H7" s="20" t="n">
         <v>1</v>
       </c>
@@ -3487,16 +3467,16 @@
         <v/>
       </c>
       <c r="AH7" s="33" t="n">
-        <v>1170652</v>
+        <v>3890964</v>
       </c>
       <c r="AI7" s="34" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="AJ7" s="34" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>med-low</t>
         </is>
       </c>
       <c r="AK7" s="41" t="n">
@@ -3543,52 +3523,48 @@
         <f>IF(((T7*pax_cap*load_full*IF(ABS(MOD(ABS((L7*M7*revleg_full)),1)-0.5)&lt;1E-9,2*ROUND((L7*M7*revleg_full)/2,0),ROUND((L7*M7*revleg_full),0)))-(((battery/range_nm)*D7*IF(ABS(MOD(ABS((L7*M7*revleg_full)),1)-0.5)&lt;1E-9,2*ROUND((L7*M7*revleg_full)/2,0),ROUND((L7*M7*revleg_full),0))*VLOOKUP(B7,country_opex,3,FALSE))+W7+X7+Y7+Z7+AA7))&lt;=0,"",VLOOKUP(B7,country_opex,7,FALSE)/((T7*pax_cap*load_full*IF(ABS(MOD(ABS((L7*M7*revleg_full)),1)-0.5)&lt;1E-9,2*ROUND((L7*M7*revleg_full)/2,0),ROUND((L7*M7*revleg_full),0)))-(((battery/range_nm)*D7*IF(ABS(MOD(ABS((L7*M7*revleg_full)),1)-0.5)&lt;1E-9,2*ROUND((L7*M7*revleg_full)/2,0),ROUND((L7*M7*revleg_full),0))*VLOOKUP(B7,country_opex,3,FALSE))+W7+X7+Y7+Z7+AA7)))</f>
         <v/>
       </c>
-      <c r="AY7" s="46" t="inlineStr">
-        <is>
-          <t>https://barcasrio.com.br/linhas-horarios-e-tarifas/</t>
-        </is>
-      </c>
+      <c r="AY7" s="46" t="n"/>
       <c r="AZ7" s="46" t="inlineStr">
         <is>
-          <t>https://www2.agetransp.rj.gov.br/arquivos/operacao-servicos/relatorio-de-atividades/Relat%C3%B3rio%20Mensal%20de%20Atividades%20Janeiro%202024.pdf</t>
+          <t>https://www.sie.sc.gov.br/webdocs/sie/doc-tecnicos/aquaviario/ (EVTE Aquaviario RMF, Relatorio 3 - Componente Demanda; SIE-SC + BID)</t>
         </is>
       </c>
       <c r="BA7" s="34" t="inlineStr">
         <is>
-          <t>rn-00bb6ded4be5</t>
+          <t>rn-floripa-r3-PROV</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="31" t="inlineStr">
         <is>
-          <t>Mexico Caribbean</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="B8" s="31" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="C8" s="32" t="inlineStr">
         <is>
-          <t>Punta Sam ferry terminal → Terminal Martima De Isla Mujeres</t>
+          <t>Praça XV Terminal (central Rio) → Cocotá Terminal (Ilha do Governador)</t>
         </is>
       </c>
       <c r="D8" s="33" t="n">
-        <v>3.35</v>
+        <v>6</v>
       </c>
       <c r="E8" s="27" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="F8" s="34" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>T1/T2</t>
         </is>
       </c>
       <c r="G8" s="34" t="inlineStr">
         <is>
-          <t>med</t>
+          <t>med-low</t>
         </is>
       </c>
       <c r="H8" s="20" t="n">
@@ -3695,7 +3671,7 @@
         <v/>
       </c>
       <c r="AH8" s="33" t="n">
-        <v>238128</v>
+        <v>278607</v>
       </c>
       <c r="AI8" s="34" t="inlineStr">
         <is>
@@ -3753,42 +3729,52 @@
       </c>
       <c r="AY8" s="46" t="inlineStr">
         <is>
-          <t>https://www.uber.com/mx/en/ride/uber-black/</t>
+          <t>https://barcasrio.com.br/linhas-horarios-e-tarifas/</t>
         </is>
       </c>
       <c r="AZ8" s="46" t="inlineStr">
         <is>
-          <t>https://servicios.apiqroo.com.mx/estadistica/datos/informeTransbordador.php?anio=2025</t>
+          <t>https://www2.agetransp.rj.gov.br/arquivos/operacao-servicos/relatorio-de-atividades/Relat%C3%B3rio%20Mensal%20de%20Atividades%20Janeiro%202024.pdf</t>
         </is>
       </c>
       <c r="BA8" s="34" t="inlineStr">
         <is>
-          <t>ics-aa6ff40d2d</t>
+          <t>rn-369ef0eb69d9</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="31" t="inlineStr">
         <is>
-          <t>Mexico Pacific</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="B9" s="31" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="C9" s="32" t="inlineStr">
         <is>
-          <t>Palmilla → San José Del Cabo Marina</t>
+          <t>Praça XV Terminal (central Rio) → Paquetá Island Terminal</t>
         </is>
       </c>
       <c r="D9" s="33" t="n">
-        <v>3.4</v>
-      </c>
-      <c r="E9" s="27" t="n"/>
-      <c r="F9" s="34" t="n"/>
-      <c r="G9" s="34" t="n"/>
+        <v>9.199999999999999</v>
+      </c>
+      <c r="E9" s="27" t="n">
+        <v>28</v>
+      </c>
+      <c r="F9" s="34" t="inlineStr">
+        <is>
+          <t>T1/T2</t>
+        </is>
+      </c>
+      <c r="G9" s="34" t="inlineStr">
+        <is>
+          <t>med-low</t>
+        </is>
+      </c>
       <c r="H9" s="20" t="n">
         <v>1</v>
       </c>
@@ -3892,9 +3878,19 @@
         <f>((D9*P9/diesel_nmpg)*diesel_co2pg-(battery/range_nm)*D9*P9*VLOOKUP(B9,country_opex,4,FALSE))/1000</f>
         <v/>
       </c>
-      <c r="AH9" s="33" t="n"/>
-      <c r="AI9" s="34" t="n"/>
-      <c r="AJ9" s="34" t="n"/>
+      <c r="AH9" s="33" t="n">
+        <v>1170652</v>
+      </c>
+      <c r="AI9" s="34" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="AJ9" s="34" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
       <c r="AK9" s="41" t="n">
         <v>0.1</v>
       </c>
@@ -3921,7 +3917,7 @@
       <c r="AQ9" s="42" t="n"/>
       <c r="AR9" s="34" t="inlineStr">
         <is>
-          <t>Estimated</t>
+          <t>Grounded</t>
         </is>
       </c>
       <c r="AS9" s="43" t="n"/>
@@ -3939,44 +3935,52 @@
         <f>IF(((T9*pax_cap*load_full*IF(ABS(MOD(ABS((L9*M9*revleg_full)),1)-0.5)&lt;1E-9,2*ROUND((L9*M9*revleg_full)/2,0),ROUND((L9*M9*revleg_full),0)))-(((battery/range_nm)*D9*IF(ABS(MOD(ABS((L9*M9*revleg_full)),1)-0.5)&lt;1E-9,2*ROUND((L9*M9*revleg_full)/2,0),ROUND((L9*M9*revleg_full),0))*VLOOKUP(B9,country_opex,3,FALSE))+W9+X9+Y9+Z9+AA9))&lt;=0,"",VLOOKUP(B9,country_opex,7,FALSE)/((T9*pax_cap*load_full*IF(ABS(MOD(ABS((L9*M9*revleg_full)),1)-0.5)&lt;1E-9,2*ROUND((L9*M9*revleg_full)/2,0),ROUND((L9*M9*revleg_full),0)))-(((battery/range_nm)*D9*IF(ABS(MOD(ABS((L9*M9*revleg_full)),1)-0.5)&lt;1E-9,2*ROUND((L9*M9*revleg_full)/2,0),ROUND((L9*M9*revleg_full),0))*VLOOKUP(B9,country_opex,3,FALSE))+W9+X9+Y9+Z9+AA9)))</f>
         <v/>
       </c>
-      <c r="AY9" s="46" t="n"/>
-      <c r="AZ9" s="46" t="n"/>
+      <c r="AY9" s="46" t="inlineStr">
+        <is>
+          <t>https://barcasrio.com.br/linhas-horarios-e-tarifas/</t>
+        </is>
+      </c>
+      <c r="AZ9" s="46" t="inlineStr">
+        <is>
+          <t>https://www2.agetransp.rj.gov.br/arquivos/operacao-servicos/relatorio-de-atividades/Relat%C3%B3rio%20Mensal%20de%20Atividades%20Janeiro%202024.pdf</t>
+        </is>
+      </c>
       <c r="BA9" s="34" t="inlineStr">
         <is>
-          <t>ics-b5861451fb</t>
+          <t>rn-00bb6ded4be5</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="31" t="inlineStr">
         <is>
-          <t>Mexico Caribbean</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="B10" s="31" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="C10" s="32" t="inlineStr">
         <is>
-          <t>Terminal Maritima Puerto Juarez → Terminal Martima De Isla Mujeres</t>
+          <t>Angra dos Reis Terminal (Costa Verde) → Abraão Terminal (Ilha Grande)</t>
         </is>
       </c>
       <c r="D10" s="33" t="n">
-        <v>5.27</v>
+        <v>13</v>
       </c>
       <c r="E10" s="27" t="n">
         <v>30</v>
       </c>
       <c r="F10" s="34" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="G10" s="34" t="inlineStr">
         <is>
-          <t>med</t>
+          <t>high</t>
         </is>
       </c>
       <c r="H10" s="20" t="n">
@@ -4083,7 +4087,7 @@
         <v/>
       </c>
       <c r="AH10" s="33" t="n">
-        <v>5458304</v>
+        <v>207993</v>
       </c>
       <c r="AI10" s="34" t="inlineStr">
         <is>
@@ -4141,17 +4145,17 @@
       </c>
       <c r="AY10" s="46" t="inlineStr">
         <is>
-          <t>https://www.uber.com/mx/en/ride/uber-black/</t>
+          <t>AGETRANSP / CCR Barcas Costa Verde published tariff</t>
         </is>
       </c>
       <c r="AZ10" s="46" t="inlineStr">
         <is>
-          <t>https://servicios.apiqroo.com.mx/estadistica/datos/informeRutaPasaje.php?anio=2025</t>
+          <t>https://www2.agetransp.rj.gov.br/arquivos/operacao-servicos/relatorio-de-atividades/Relat%C3%B3rio%20Mensal%20de%20Atividades%20Janeiro%202024.pdf</t>
         </is>
       </c>
       <c r="BA10" s="34" t="inlineStr">
         <is>
-          <t>ics-413f51cd44</t>
+          <t>rn-angra-abraao-PROV</t>
         </is>
       </c>
     </row>
@@ -4168,15 +4172,25 @@
       </c>
       <c r="C11" s="32" t="inlineStr">
         <is>
-          <t>Ultramar → Terminal Martima De Isla Mujeres</t>
+          <t>Punta Sam ferry terminal → Terminal Martima De Isla Mujeres</t>
         </is>
       </c>
       <c r="D11" s="33" t="n">
-        <v>5.49</v>
-      </c>
-      <c r="E11" s="27" t="n"/>
-      <c r="F11" s="34" t="n"/>
-      <c r="G11" s="34" t="n"/>
+        <v>3.35</v>
+      </c>
+      <c r="E11" s="27" t="n">
+        <v>30</v>
+      </c>
+      <c r="F11" s="34" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="G11" s="34" t="inlineStr">
+        <is>
+          <t>med</t>
+        </is>
+      </c>
       <c r="H11" s="20" t="n">
         <v>1</v>
       </c>
@@ -4280,9 +4294,19 @@
         <f>((D11*P11/diesel_nmpg)*diesel_co2pg-(battery/range_nm)*D11*P11*VLOOKUP(B11,country_opex,4,FALSE))/1000</f>
         <v/>
       </c>
-      <c r="AH11" s="33" t="n"/>
-      <c r="AI11" s="34" t="n"/>
-      <c r="AJ11" s="34" t="n"/>
+      <c r="AH11" s="33" t="n">
+        <v>238128</v>
+      </c>
+      <c r="AI11" s="34" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="AJ11" s="34" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
       <c r="AK11" s="41" t="n">
         <v>0.1</v>
       </c>
@@ -4309,7 +4333,7 @@
       <c r="AQ11" s="42" t="n"/>
       <c r="AR11" s="34" t="inlineStr">
         <is>
-          <t>Estimated</t>
+          <t>Grounded</t>
         </is>
       </c>
       <c r="AS11" s="43" t="n"/>
@@ -4327,18 +4351,26 @@
         <f>IF(((T11*pax_cap*load_full*IF(ABS(MOD(ABS((L11*M11*revleg_full)),1)-0.5)&lt;1E-9,2*ROUND((L11*M11*revleg_full)/2,0),ROUND((L11*M11*revleg_full),0)))-(((battery/range_nm)*D11*IF(ABS(MOD(ABS((L11*M11*revleg_full)),1)-0.5)&lt;1E-9,2*ROUND((L11*M11*revleg_full)/2,0),ROUND((L11*M11*revleg_full),0))*VLOOKUP(B11,country_opex,3,FALSE))+W11+X11+Y11+Z11+AA11))&lt;=0,"",VLOOKUP(B11,country_opex,7,FALSE)/((T11*pax_cap*load_full*IF(ABS(MOD(ABS((L11*M11*revleg_full)),1)-0.5)&lt;1E-9,2*ROUND((L11*M11*revleg_full)/2,0),ROUND((L11*M11*revleg_full),0)))-(((battery/range_nm)*D11*IF(ABS(MOD(ABS((L11*M11*revleg_full)),1)-0.5)&lt;1E-9,2*ROUND((L11*M11*revleg_full)/2,0),ROUND((L11*M11*revleg_full),0))*VLOOKUP(B11,country_opex,3,FALSE))+W11+X11+Y11+Z11+AA11)))</f>
         <v/>
       </c>
-      <c r="AY11" s="46" t="n"/>
-      <c r="AZ11" s="46" t="n"/>
+      <c r="AY11" s="46" t="inlineStr">
+        <is>
+          <t>https://www.uber.com/mx/en/ride/uber-black/</t>
+        </is>
+      </c>
+      <c r="AZ11" s="46" t="inlineStr">
+        <is>
+          <t>https://servicios.apiqroo.com.mx/estadistica/datos/informeTransbordador.php?anio=2025</t>
+        </is>
+      </c>
       <c r="BA11" s="34" t="inlineStr">
         <is>
-          <t>ics-03e3853317</t>
+          <t>ics-aa6ff40d2d</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="31" t="inlineStr">
         <is>
-          <t>Mexico Caribbean</t>
+          <t>Mexico Pacific</t>
         </is>
       </c>
       <c r="B12" s="31" t="inlineStr">
@@ -4348,25 +4380,15 @@
       </c>
       <c r="C12" s="32" t="inlineStr">
         <is>
-          <t>Muelle Fiscal Playa del Carmen → Passenger Ferry Ultramar Cozumel</t>
+          <t>Palmilla → San José Del Cabo Marina</t>
         </is>
       </c>
       <c r="D12" s="33" t="n">
-        <v>9.529999999999999</v>
-      </c>
-      <c r="E12" s="27" t="n">
-        <v>30</v>
-      </c>
-      <c r="F12" s="34" t="inlineStr">
-        <is>
-          <t>T2</t>
-        </is>
-      </c>
-      <c r="G12" s="34" t="inlineStr">
-        <is>
-          <t>med</t>
-        </is>
-      </c>
+        <v>3.4</v>
+      </c>
+      <c r="E12" s="27" t="n"/>
+      <c r="F12" s="34" t="n"/>
+      <c r="G12" s="34" t="n"/>
       <c r="H12" s="20" t="n">
         <v>1</v>
       </c>
@@ -4470,19 +4492,9 @@
         <f>((D12*P12/diesel_nmpg)*diesel_co2pg-(battery/range_nm)*D12*P12*VLOOKUP(B12,country_opex,4,FALSE))/1000</f>
         <v/>
       </c>
-      <c r="AH12" s="33" t="n">
-        <v>3853770</v>
-      </c>
-      <c r="AI12" s="34" t="inlineStr">
-        <is>
-          <t>T1</t>
-        </is>
-      </c>
-      <c r="AJ12" s="34" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
+      <c r="AH12" s="33" t="n"/>
+      <c r="AI12" s="34" t="n"/>
+      <c r="AJ12" s="34" t="n"/>
       <c r="AK12" s="41" t="n">
         <v>0.1</v>
       </c>
@@ -4509,7 +4521,7 @@
       <c r="AQ12" s="42" t="n"/>
       <c r="AR12" s="34" t="inlineStr">
         <is>
-          <t>Grounded</t>
+          <t>Estimated</t>
         </is>
       </c>
       <c r="AS12" s="43" t="n"/>
@@ -4527,26 +4539,18 @@
         <f>IF(((T12*pax_cap*load_full*IF(ABS(MOD(ABS((L12*M12*revleg_full)),1)-0.5)&lt;1E-9,2*ROUND((L12*M12*revleg_full)/2,0),ROUND((L12*M12*revleg_full),0)))-(((battery/range_nm)*D12*IF(ABS(MOD(ABS((L12*M12*revleg_full)),1)-0.5)&lt;1E-9,2*ROUND((L12*M12*revleg_full)/2,0),ROUND((L12*M12*revleg_full),0))*VLOOKUP(B12,country_opex,3,FALSE))+W12+X12+Y12+Z12+AA12))&lt;=0,"",VLOOKUP(B12,country_opex,7,FALSE)/((T12*pax_cap*load_full*IF(ABS(MOD(ABS((L12*M12*revleg_full)),1)-0.5)&lt;1E-9,2*ROUND((L12*M12*revleg_full)/2,0),ROUND((L12*M12*revleg_full),0)))-(((battery/range_nm)*D12*IF(ABS(MOD(ABS((L12*M12*revleg_full)),1)-0.5)&lt;1E-9,2*ROUND((L12*M12*revleg_full)/2,0),ROUND((L12*M12*revleg_full),0))*VLOOKUP(B12,country_opex,3,FALSE))+W12+X12+Y12+Z12+AA12)))</f>
         <v/>
       </c>
-      <c r="AY12" s="46" t="inlineStr">
-        <is>
-          <t>https://www.uber.com/mx/en/ride/uber-black/</t>
-        </is>
-      </c>
-      <c r="AZ12" s="46" t="inlineStr">
-        <is>
-          <t>https://servicios.apiqroo.com.mx/estadistica/datos/informeRutaPasaje.php?anio=2025</t>
-        </is>
-      </c>
+      <c r="AY12" s="46" t="n"/>
+      <c r="AZ12" s="46" t="n"/>
       <c r="BA12" s="34" t="inlineStr">
         <is>
-          <t>ics-dd1d814699</t>
+          <t>ics-b5861451fb</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="31" t="inlineStr">
         <is>
-          <t>Mexico Pacific</t>
+          <t>Mexico Caribbean</t>
         </is>
       </c>
       <c r="B13" s="31" t="inlineStr">
@@ -4556,15 +4560,25 @@
       </c>
       <c r="C13" s="32" t="inlineStr">
         <is>
-          <t>Puerto Vallarta &amp; Riviera Nayarit → Punta De Mita</t>
+          <t>Terminal Maritima Puerto Juarez → Terminal Martima De Isla Mujeres</t>
         </is>
       </c>
       <c r="D13" s="33" t="n">
-        <v>9.9</v>
-      </c>
-      <c r="E13" s="27" t="n"/>
-      <c r="F13" s="34" t="n"/>
-      <c r="G13" s="34" t="n"/>
+        <v>5.27</v>
+      </c>
+      <c r="E13" s="27" t="n">
+        <v>30</v>
+      </c>
+      <c r="F13" s="34" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="G13" s="34" t="inlineStr">
+        <is>
+          <t>med</t>
+        </is>
+      </c>
       <c r="H13" s="20" t="n">
         <v>1</v>
       </c>
@@ -4668,9 +4682,19 @@
         <f>((D13*P13/diesel_nmpg)*diesel_co2pg-(battery/range_nm)*D13*P13*VLOOKUP(B13,country_opex,4,FALSE))/1000</f>
         <v/>
       </c>
-      <c r="AH13" s="33" t="n"/>
-      <c r="AI13" s="34" t="n"/>
-      <c r="AJ13" s="34" t="n"/>
+      <c r="AH13" s="33" t="n">
+        <v>5458304</v>
+      </c>
+      <c r="AI13" s="34" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="AJ13" s="34" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
       <c r="AK13" s="41" t="n">
         <v>0.1</v>
       </c>
@@ -4697,7 +4721,7 @@
       <c r="AQ13" s="42" t="n"/>
       <c r="AR13" s="34" t="inlineStr">
         <is>
-          <t>Estimated</t>
+          <t>Grounded</t>
         </is>
       </c>
       <c r="AS13" s="43" t="n"/>
@@ -4715,18 +4739,26 @@
         <f>IF(((T13*pax_cap*load_full*IF(ABS(MOD(ABS((L13*M13*revleg_full)),1)-0.5)&lt;1E-9,2*ROUND((L13*M13*revleg_full)/2,0),ROUND((L13*M13*revleg_full),0)))-(((battery/range_nm)*D13*IF(ABS(MOD(ABS((L13*M13*revleg_full)),1)-0.5)&lt;1E-9,2*ROUND((L13*M13*revleg_full)/2,0),ROUND((L13*M13*revleg_full),0))*VLOOKUP(B13,country_opex,3,FALSE))+W13+X13+Y13+Z13+AA13))&lt;=0,"",VLOOKUP(B13,country_opex,7,FALSE)/((T13*pax_cap*load_full*IF(ABS(MOD(ABS((L13*M13*revleg_full)),1)-0.5)&lt;1E-9,2*ROUND((L13*M13*revleg_full)/2,0),ROUND((L13*M13*revleg_full),0)))-(((battery/range_nm)*D13*IF(ABS(MOD(ABS((L13*M13*revleg_full)),1)-0.5)&lt;1E-9,2*ROUND((L13*M13*revleg_full)/2,0),ROUND((L13*M13*revleg_full),0))*VLOOKUP(B13,country_opex,3,FALSE))+W13+X13+Y13+Z13+AA13)))</f>
         <v/>
       </c>
-      <c r="AY13" s="46" t="n"/>
-      <c r="AZ13" s="46" t="n"/>
+      <c r="AY13" s="46" t="inlineStr">
+        <is>
+          <t>https://www.uber.com/mx/en/ride/uber-black/</t>
+        </is>
+      </c>
+      <c r="AZ13" s="46" t="inlineStr">
+        <is>
+          <t>https://servicios.apiqroo.com.mx/estadistica/datos/informeRutaPasaje.php?anio=2025</t>
+        </is>
+      </c>
       <c r="BA13" s="34" t="inlineStr">
         <is>
-          <t>ics-de6758216f</t>
+          <t>ics-413f51cd44</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="31" t="inlineStr">
         <is>
-          <t>Mexico Pacific</t>
+          <t>Mexico Caribbean</t>
         </is>
       </c>
       <c r="B14" s="31" t="inlineStr">
@@ -4736,25 +4768,15 @@
       </c>
       <c r="C14" s="32" t="inlineStr">
         <is>
-          <t>Puerto Vallarta &amp; Riviera Nayarit → Yelapa</t>
+          <t>Ultramar → Terminal Martima De Isla Mujeres</t>
         </is>
       </c>
       <c r="D14" s="33" t="n">
-        <v>14.5</v>
-      </c>
-      <c r="E14" s="27" t="n">
-        <v>18.19</v>
-      </c>
-      <c r="F14" s="34" t="inlineStr">
-        <is>
-          <t>T2</t>
-        </is>
-      </c>
-      <c r="G14" s="34" t="inlineStr">
-        <is>
-          <t>med</t>
-        </is>
-      </c>
+        <v>5.49</v>
+      </c>
+      <c r="E14" s="27" t="n"/>
+      <c r="F14" s="34" t="n"/>
+      <c r="G14" s="34" t="n"/>
       <c r="H14" s="20" t="n">
         <v>1</v>
       </c>
@@ -4905,22 +4927,18 @@
         <f>IF(((T14*pax_cap*load_full*IF(ABS(MOD(ABS((L14*M14*revleg_full)),1)-0.5)&lt;1E-9,2*ROUND((L14*M14*revleg_full)/2,0),ROUND((L14*M14*revleg_full),0)))-(((battery/range_nm)*D14*IF(ABS(MOD(ABS((L14*M14*revleg_full)),1)-0.5)&lt;1E-9,2*ROUND((L14*M14*revleg_full)/2,0),ROUND((L14*M14*revleg_full),0))*VLOOKUP(B14,country_opex,3,FALSE))+W14+X14+Y14+Z14+AA14))&lt;=0,"",VLOOKUP(B14,country_opex,7,FALSE)/((T14*pax_cap*load_full*IF(ABS(MOD(ABS((L14*M14*revleg_full)),1)-0.5)&lt;1E-9,2*ROUND((L14*M14*revleg_full)/2,0),ROUND((L14*M14*revleg_full),0)))-(((battery/range_nm)*D14*IF(ABS(MOD(ABS((L14*M14*revleg_full)),1)-0.5)&lt;1E-9,2*ROUND((L14*M14*revleg_full)/2,0),ROUND((L14*M14*revleg_full),0))*VLOOKUP(B14,country_opex,3,FALSE))+W14+X14+Y14+Z14+AA14)))</f>
         <v/>
       </c>
-      <c r="AY14" s="46" t="inlineStr">
-        <is>
-          <t>https://www.yelapa.info/transport1.html</t>
-        </is>
-      </c>
+      <c r="AY14" s="46" t="n"/>
       <c r="AZ14" s="46" t="n"/>
       <c r="BA14" s="34" t="inlineStr">
         <is>
-          <t>ics-89a8844858</t>
+          <t>ics-03e3853317</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="31" t="inlineStr">
         <is>
-          <t>Mexico Pacific</t>
+          <t>Mexico Caribbean</t>
         </is>
       </c>
       <c r="B15" s="31" t="inlineStr">
@@ -4930,15 +4948,25 @@
       </c>
       <c r="C15" s="32" t="inlineStr">
         <is>
-          <t>Cabo San Lucas Marina → Los Cabos, Baja Sur</t>
+          <t>Muelle Fiscal Playa del Carmen → Passenger Ferry Ultramar Cozumel</t>
         </is>
       </c>
       <c r="D15" s="33" t="n">
-        <v>17</v>
-      </c>
-      <c r="E15" s="27" t="n"/>
-      <c r="F15" s="34" t="n"/>
-      <c r="G15" s="34" t="n"/>
+        <v>9.529999999999999</v>
+      </c>
+      <c r="E15" s="27" t="n">
+        <v>30</v>
+      </c>
+      <c r="F15" s="34" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="G15" s="34" t="inlineStr">
+        <is>
+          <t>med</t>
+        </is>
+      </c>
       <c r="H15" s="20" t="n">
         <v>1</v>
       </c>
@@ -5042,9 +5070,19 @@
         <f>((D15*P15/diesel_nmpg)*diesel_co2pg-(battery/range_nm)*D15*P15*VLOOKUP(B15,country_opex,4,FALSE))/1000</f>
         <v/>
       </c>
-      <c r="AH15" s="33" t="n"/>
-      <c r="AI15" s="34" t="n"/>
-      <c r="AJ15" s="34" t="n"/>
+      <c r="AH15" s="33" t="n">
+        <v>3853770</v>
+      </c>
+      <c r="AI15" s="34" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="AJ15" s="34" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
       <c r="AK15" s="41" t="n">
         <v>0.1</v>
       </c>
@@ -5071,7 +5109,7 @@
       <c r="AQ15" s="42" t="n"/>
       <c r="AR15" s="34" t="inlineStr">
         <is>
-          <t>Estimated</t>
+          <t>Grounded</t>
         </is>
       </c>
       <c r="AS15" s="43" t="n"/>
@@ -5089,184 +5127,746 @@
         <f>IF(((T15*pax_cap*load_full*IF(ABS(MOD(ABS((L15*M15*revleg_full)),1)-0.5)&lt;1E-9,2*ROUND((L15*M15*revleg_full)/2,0),ROUND((L15*M15*revleg_full),0)))-(((battery/range_nm)*D15*IF(ABS(MOD(ABS((L15*M15*revleg_full)),1)-0.5)&lt;1E-9,2*ROUND((L15*M15*revleg_full)/2,0),ROUND((L15*M15*revleg_full),0))*VLOOKUP(B15,country_opex,3,FALSE))+W15+X15+Y15+Z15+AA15))&lt;=0,"",VLOOKUP(B15,country_opex,7,FALSE)/((T15*pax_cap*load_full*IF(ABS(MOD(ABS((L15*M15*revleg_full)),1)-0.5)&lt;1E-9,2*ROUND((L15*M15*revleg_full)/2,0),ROUND((L15*M15*revleg_full),0)))-(((battery/range_nm)*D15*IF(ABS(MOD(ABS((L15*M15*revleg_full)),1)-0.5)&lt;1E-9,2*ROUND((L15*M15*revleg_full)/2,0),ROUND((L15*M15*revleg_full),0))*VLOOKUP(B15,country_opex,3,FALSE))+W15+X15+Y15+Z15+AA15)))</f>
         <v/>
       </c>
-      <c r="AY15" s="46" t="n"/>
-      <c r="AZ15" s="46" t="n"/>
+      <c r="AY15" s="46" t="inlineStr">
+        <is>
+          <t>https://www.uber.com/mx/en/ride/uber-black/</t>
+        </is>
+      </c>
+      <c r="AZ15" s="46" t="inlineStr">
+        <is>
+          <t>https://servicios.apiqroo.com.mx/estadistica/datos/informeRutaPasaje.php?anio=2025</t>
+        </is>
+      </c>
       <c r="BA15" s="34" t="inlineStr">
         <is>
+          <t>ics-dd1d814699</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="31" t="inlineStr">
+        <is>
+          <t>Mexico Pacific</t>
+        </is>
+      </c>
+      <c r="B16" s="31" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="C16" s="32" t="inlineStr">
+        <is>
+          <t>Puerto Vallarta &amp; Riviera Nayarit → Punta De Mita</t>
+        </is>
+      </c>
+      <c r="D16" s="33" t="n">
+        <v>9.9</v>
+      </c>
+      <c r="E16" s="27" t="n"/>
+      <c r="F16" s="34" t="n"/>
+      <c r="G16" s="34" t="n"/>
+      <c r="H16" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="I16" s="35">
+        <f>60*D16/cruise_kt</f>
+        <v/>
+      </c>
+      <c r="J16" s="35">
+        <f>IF(B16="South Korea",D16/korea_charge_range_nm*korea_full_range_charge_min,0)</f>
+        <v/>
+      </c>
+      <c r="K16" s="35">
+        <f>IF(B16="South Korea",I16+korea_turn_min+korea_dwell_min+J16,I16+turn_min+dwell_min)</f>
+        <v/>
+      </c>
+      <c r="L16" s="36">
+        <f>IF(B16="South Korea",FLOOR(60*korea_service_hr/K16,1),MIN(15,FLOOR(60*service_hr/K16,1)))</f>
+        <v/>
+      </c>
+      <c r="M16" s="36">
+        <f>IF(ABS(MOD(ABS((365*mech_uptime*H16)),1)-0.5)&lt;1E-9,2*ROUND((365*mech_uptime*H16)/2,0),ROUND((365*mech_uptime*H16),0))</f>
+        <v/>
+      </c>
+      <c r="N16" s="37">
+        <f>mech_uptime</f>
+        <v/>
+      </c>
+      <c r="O16" s="37">
+        <f>IF(AND(B16="South Korea",scenario="MID"),korea_mid_revleg,revleg_sel)</f>
+        <v/>
+      </c>
+      <c r="P16" s="36">
+        <f>IF(ABS(MOD(ABS((L16*M16*O16)),1)-0.5)&lt;1E-9,2*ROUND((L16*M16*O16)/2,0),ROUND((L16*M16*O16),0))</f>
+        <v/>
+      </c>
+      <c r="Q16" s="37">
+        <f>IF(AND(B16="South Korea",scenario="MID"),korea_mid_load,load_sel)</f>
+        <v/>
+      </c>
+      <c r="R16" s="38">
+        <f>pax_cap*Q16</f>
+        <v/>
+      </c>
+      <c r="S16" s="36">
+        <f>R16*P16</f>
+        <v/>
+      </c>
+      <c r="T16" s="39">
+        <f>E16*discount</f>
+        <v/>
+      </c>
+      <c r="U16" s="40">
+        <f>T16*S16</f>
+        <v/>
+      </c>
+      <c r="V16" s="40">
+        <f>(battery/range_nm)*D16*P16*VLOOKUP(B16,country_opex,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="W16" s="40">
+        <f>VLOOKUP(B16,country_opex,2,FALSE)*crew_factor</f>
+        <v/>
+      </c>
+      <c r="X16" s="40">
+        <f>VLOOKUP(B16,country_opex,5,FALSE)</f>
+        <v/>
+      </c>
+      <c r="Y16" s="40">
+        <f>maint</f>
+        <v/>
+      </c>
+      <c r="Z16" s="40">
+        <f>VLOOKUP(B16,country_opex,7,FALSE)*ins_pct</f>
+        <v/>
+      </c>
+      <c r="AA16" s="40">
+        <f>charge_berth</f>
+        <v/>
+      </c>
+      <c r="AB16" s="40">
+        <f>V16+W16+X16+Y16+Z16+AA16</f>
+        <v/>
+      </c>
+      <c r="AC16" s="40">
+        <f>VLOOKUP(B16,country_opex,7,FALSE)/dep_years</f>
+        <v/>
+      </c>
+      <c r="AD16" s="40">
+        <f>U16-AB16</f>
+        <v/>
+      </c>
+      <c r="AE16" s="37">
+        <f>IF(U16=0,"",AD16/U16)</f>
+        <v/>
+      </c>
+      <c r="AF16" s="38">
+        <f>IF(AD16&lt;=0,"",VLOOKUP(B16,country_opex,7,FALSE)/AD16)</f>
+        <v/>
+      </c>
+      <c r="AG16" s="35">
+        <f>((D16*P16/diesel_nmpg)*diesel_co2pg-(battery/range_nm)*D16*P16*VLOOKUP(B16,country_opex,4,FALSE))/1000</f>
+        <v/>
+      </c>
+      <c r="AH16" s="33" t="n"/>
+      <c r="AI16" s="34" t="n"/>
+      <c r="AJ16" s="34" t="n"/>
+      <c r="AK16" s="41" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="AL16" s="36">
+        <f>IF(AH16="","",AH16*AK16)</f>
+        <v/>
+      </c>
+      <c r="AM16" s="36">
+        <f>IF(OR(AH16="",S16=0),"",MIN(IF(AU16="",9.9E+99,AU16),FLOOR(AL16/S16,1)))</f>
+        <v/>
+      </c>
+      <c r="AN16" s="40">
+        <f>IF(AM16="","",AM16*IF(ABS(MOD(ABS((U16)),1)-0.5)&lt;1E-9,2*ROUND((U16)/2,0),ROUND((U16),0)))</f>
+        <v/>
+      </c>
+      <c r="AO16" s="38">
+        <f>IF(OR(AH16="",S16=0),"",MIN(IF(AU16="",9.9E+99,AU16),AL16/S16))</f>
+        <v/>
+      </c>
+      <c r="AP16" s="40">
+        <f>IF(AO16="","",AO16*IF(B16="South Korea",IF(ABS(MOD(ABS((U16)),1)-0.5)&lt;1E-9,2*ROUND((U16)/2,0),ROUND((U16),0)),U16))</f>
+        <v/>
+      </c>
+      <c r="AQ16" s="42" t="n"/>
+      <c r="AR16" s="34" t="inlineStr">
+        <is>
+          <t>Estimated</t>
+        </is>
+      </c>
+      <c r="AS16" s="43" t="n"/>
+      <c r="AT16" s="43" t="n"/>
+      <c r="AU16" s="44" t="n"/>
+      <c r="AV16" s="45">
+        <f>IF(((T16*pax_cap*load_thin*IF(ABS(MOD(ABS((L16*M16*revleg_thin)),1)-0.5)&lt;1E-9,2*ROUND((L16*M16*revleg_thin)/2,0),ROUND((L16*M16*revleg_thin),0)))-(((battery/range_nm)*D16*IF(ABS(MOD(ABS((L16*M16*revleg_thin)),1)-0.5)&lt;1E-9,2*ROUND((L16*M16*revleg_thin)/2,0),ROUND((L16*M16*revleg_thin),0))*VLOOKUP(B16,country_opex,3,FALSE))+W16+X16+Y16+Z16+AA16))&lt;=0,"",VLOOKUP(B16,country_opex,7,FALSE)/((T16*pax_cap*load_thin*IF(ABS(MOD(ABS((L16*M16*revleg_thin)),1)-0.5)&lt;1E-9,2*ROUND((L16*M16*revleg_thin)/2,0),ROUND((L16*M16*revleg_thin),0)))-(((battery/range_nm)*D16*IF(ABS(MOD(ABS((L16*M16*revleg_thin)),1)-0.5)&lt;1E-9,2*ROUND((L16*M16*revleg_thin)/2,0),ROUND((L16*M16*revleg_thin),0))*VLOOKUP(B16,country_opex,3,FALSE))+W16+X16+Y16+Z16+AA16)))</f>
+        <v/>
+      </c>
+      <c r="AW16" s="45">
+        <f>IF(((T16*pax_cap*IF(B16="South Korea",korea_mid_load,load_mid)*IF(ABS(MOD(ABS((L16*M16*IF(B16="South Korea",korea_mid_revleg,revleg_mid))),1)-0.5)&lt;1E-9,2*ROUND((L16*M16*IF(B16="South Korea",korea_mid_revleg,revleg_mid))/2,0),ROUND((L16*M16*IF(B16="South Korea",korea_mid_revleg,revleg_mid)),0)))-(((battery/range_nm)*D16*IF(ABS(MOD(ABS((L16*M16*IF(B16="South Korea",korea_mid_revleg,revleg_mid))),1)-0.5)&lt;1E-9,2*ROUND((L16*M16*IF(B16="South Korea",korea_mid_revleg,revleg_mid))/2,0),ROUND((L16*M16*IF(B16="South Korea",korea_mid_revleg,revleg_mid)),0))*VLOOKUP(B16,country_opex,3,FALSE))+W16+X16+Y16+Z16+AA16))&lt;=0,"",VLOOKUP(B16,country_opex,7,FALSE)/((T16*pax_cap*IF(B16="South Korea",korea_mid_load,load_mid)*IF(ABS(MOD(ABS((L16*M16*IF(B16="South Korea",korea_mid_revleg,revleg_mid))),1)-0.5)&lt;1E-9,2*ROUND((L16*M16*IF(B16="South Korea",korea_mid_revleg,revleg_mid))/2,0),ROUND((L16*M16*IF(B16="South Korea",korea_mid_revleg,revleg_mid)),0)))-(((battery/range_nm)*D16*IF(ABS(MOD(ABS((L16*M16*IF(B16="South Korea",korea_mid_revleg,revleg_mid))),1)-0.5)&lt;1E-9,2*ROUND((L16*M16*IF(B16="South Korea",korea_mid_revleg,revleg_mid))/2,0),ROUND((L16*M16*IF(B16="South Korea",korea_mid_revleg,revleg_mid)),0))*VLOOKUP(B16,country_opex,3,FALSE))+W16+X16+Y16+Z16+AA16)))</f>
+        <v/>
+      </c>
+      <c r="AX16" s="45">
+        <f>IF(((T16*pax_cap*load_full*IF(ABS(MOD(ABS((L16*M16*revleg_full)),1)-0.5)&lt;1E-9,2*ROUND((L16*M16*revleg_full)/2,0),ROUND((L16*M16*revleg_full),0)))-(((battery/range_nm)*D16*IF(ABS(MOD(ABS((L16*M16*revleg_full)),1)-0.5)&lt;1E-9,2*ROUND((L16*M16*revleg_full)/2,0),ROUND((L16*M16*revleg_full),0))*VLOOKUP(B16,country_opex,3,FALSE))+W16+X16+Y16+Z16+AA16))&lt;=0,"",VLOOKUP(B16,country_opex,7,FALSE)/((T16*pax_cap*load_full*IF(ABS(MOD(ABS((L16*M16*revleg_full)),1)-0.5)&lt;1E-9,2*ROUND((L16*M16*revleg_full)/2,0),ROUND((L16*M16*revleg_full),0)))-(((battery/range_nm)*D16*IF(ABS(MOD(ABS((L16*M16*revleg_full)),1)-0.5)&lt;1E-9,2*ROUND((L16*M16*revleg_full)/2,0),ROUND((L16*M16*revleg_full),0))*VLOOKUP(B16,country_opex,3,FALSE))+W16+X16+Y16+Z16+AA16)))</f>
+        <v/>
+      </c>
+      <c r="AY16" s="46" t="n"/>
+      <c r="AZ16" s="46" t="n"/>
+      <c r="BA16" s="34" t="inlineStr">
+        <is>
+          <t>ics-de6758216f</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="31" t="inlineStr">
+        <is>
+          <t>Mexico Pacific</t>
+        </is>
+      </c>
+      <c r="B17" s="31" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="C17" s="32" t="inlineStr">
+        <is>
+          <t>Puerto Vallarta &amp; Riviera Nayarit → Yelapa</t>
+        </is>
+      </c>
+      <c r="D17" s="33" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="E17" s="27" t="n">
+        <v>18.19</v>
+      </c>
+      <c r="F17" s="34" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="G17" s="34" t="inlineStr">
+        <is>
+          <t>med</t>
+        </is>
+      </c>
+      <c r="H17" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="I17" s="35">
+        <f>60*D17/cruise_kt</f>
+        <v/>
+      </c>
+      <c r="J17" s="35">
+        <f>IF(B17="South Korea",D17/korea_charge_range_nm*korea_full_range_charge_min,0)</f>
+        <v/>
+      </c>
+      <c r="K17" s="35">
+        <f>IF(B17="South Korea",I17+korea_turn_min+korea_dwell_min+J17,I17+turn_min+dwell_min)</f>
+        <v/>
+      </c>
+      <c r="L17" s="36">
+        <f>IF(B17="South Korea",FLOOR(60*korea_service_hr/K17,1),MIN(15,FLOOR(60*service_hr/K17,1)))</f>
+        <v/>
+      </c>
+      <c r="M17" s="36">
+        <f>IF(ABS(MOD(ABS((365*mech_uptime*H17)),1)-0.5)&lt;1E-9,2*ROUND((365*mech_uptime*H17)/2,0),ROUND((365*mech_uptime*H17),0))</f>
+        <v/>
+      </c>
+      <c r="N17" s="37">
+        <f>mech_uptime</f>
+        <v/>
+      </c>
+      <c r="O17" s="37">
+        <f>IF(AND(B17="South Korea",scenario="MID"),korea_mid_revleg,revleg_sel)</f>
+        <v/>
+      </c>
+      <c r="P17" s="36">
+        <f>IF(ABS(MOD(ABS((L17*M17*O17)),1)-0.5)&lt;1E-9,2*ROUND((L17*M17*O17)/2,0),ROUND((L17*M17*O17),0))</f>
+        <v/>
+      </c>
+      <c r="Q17" s="37">
+        <f>IF(AND(B17="South Korea",scenario="MID"),korea_mid_load,load_sel)</f>
+        <v/>
+      </c>
+      <c r="R17" s="38">
+        <f>pax_cap*Q17</f>
+        <v/>
+      </c>
+      <c r="S17" s="36">
+        <f>R17*P17</f>
+        <v/>
+      </c>
+      <c r="T17" s="39">
+        <f>E17*discount</f>
+        <v/>
+      </c>
+      <c r="U17" s="40">
+        <f>T17*S17</f>
+        <v/>
+      </c>
+      <c r="V17" s="40">
+        <f>(battery/range_nm)*D17*P17*VLOOKUP(B17,country_opex,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="W17" s="40">
+        <f>VLOOKUP(B17,country_opex,2,FALSE)*crew_factor</f>
+        <v/>
+      </c>
+      <c r="X17" s="40">
+        <f>VLOOKUP(B17,country_opex,5,FALSE)</f>
+        <v/>
+      </c>
+      <c r="Y17" s="40">
+        <f>maint</f>
+        <v/>
+      </c>
+      <c r="Z17" s="40">
+        <f>VLOOKUP(B17,country_opex,7,FALSE)*ins_pct</f>
+        <v/>
+      </c>
+      <c r="AA17" s="40">
+        <f>charge_berth</f>
+        <v/>
+      </c>
+      <c r="AB17" s="40">
+        <f>V17+W17+X17+Y17+Z17+AA17</f>
+        <v/>
+      </c>
+      <c r="AC17" s="40">
+        <f>VLOOKUP(B17,country_opex,7,FALSE)/dep_years</f>
+        <v/>
+      </c>
+      <c r="AD17" s="40">
+        <f>U17-AB17</f>
+        <v/>
+      </c>
+      <c r="AE17" s="37">
+        <f>IF(U17=0,"",AD17/U17)</f>
+        <v/>
+      </c>
+      <c r="AF17" s="38">
+        <f>IF(AD17&lt;=0,"",VLOOKUP(B17,country_opex,7,FALSE)/AD17)</f>
+        <v/>
+      </c>
+      <c r="AG17" s="35">
+        <f>((D17*P17/diesel_nmpg)*diesel_co2pg-(battery/range_nm)*D17*P17*VLOOKUP(B17,country_opex,4,FALSE))/1000</f>
+        <v/>
+      </c>
+      <c r="AH17" s="33" t="n"/>
+      <c r="AI17" s="34" t="n"/>
+      <c r="AJ17" s="34" t="n"/>
+      <c r="AK17" s="41" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="AL17" s="36">
+        <f>IF(AH17="","",AH17*AK17)</f>
+        <v/>
+      </c>
+      <c r="AM17" s="36">
+        <f>IF(OR(AH17="",S17=0),"",MIN(IF(AU17="",9.9E+99,AU17),FLOOR(AL17/S17,1)))</f>
+        <v/>
+      </c>
+      <c r="AN17" s="40">
+        <f>IF(AM17="","",AM17*IF(ABS(MOD(ABS((U17)),1)-0.5)&lt;1E-9,2*ROUND((U17)/2,0),ROUND((U17),0)))</f>
+        <v/>
+      </c>
+      <c r="AO17" s="38">
+        <f>IF(OR(AH17="",S17=0),"",MIN(IF(AU17="",9.9E+99,AU17),AL17/S17))</f>
+        <v/>
+      </c>
+      <c r="AP17" s="40">
+        <f>IF(AO17="","",AO17*IF(B17="South Korea",IF(ABS(MOD(ABS((U17)),1)-0.5)&lt;1E-9,2*ROUND((U17)/2,0),ROUND((U17),0)),U17))</f>
+        <v/>
+      </c>
+      <c r="AQ17" s="42" t="n"/>
+      <c r="AR17" s="34" t="inlineStr">
+        <is>
+          <t>Estimated</t>
+        </is>
+      </c>
+      <c r="AS17" s="43" t="n"/>
+      <c r="AT17" s="43" t="n"/>
+      <c r="AU17" s="44" t="n"/>
+      <c r="AV17" s="45">
+        <f>IF(((T17*pax_cap*load_thin*IF(ABS(MOD(ABS((L17*M17*revleg_thin)),1)-0.5)&lt;1E-9,2*ROUND((L17*M17*revleg_thin)/2,0),ROUND((L17*M17*revleg_thin),0)))-(((battery/range_nm)*D17*IF(ABS(MOD(ABS((L17*M17*revleg_thin)),1)-0.5)&lt;1E-9,2*ROUND((L17*M17*revleg_thin)/2,0),ROUND((L17*M17*revleg_thin),0))*VLOOKUP(B17,country_opex,3,FALSE))+W17+X17+Y17+Z17+AA17))&lt;=0,"",VLOOKUP(B17,country_opex,7,FALSE)/((T17*pax_cap*load_thin*IF(ABS(MOD(ABS((L17*M17*revleg_thin)),1)-0.5)&lt;1E-9,2*ROUND((L17*M17*revleg_thin)/2,0),ROUND((L17*M17*revleg_thin),0)))-(((battery/range_nm)*D17*IF(ABS(MOD(ABS((L17*M17*revleg_thin)),1)-0.5)&lt;1E-9,2*ROUND((L17*M17*revleg_thin)/2,0),ROUND((L17*M17*revleg_thin),0))*VLOOKUP(B17,country_opex,3,FALSE))+W17+X17+Y17+Z17+AA17)))</f>
+        <v/>
+      </c>
+      <c r="AW17" s="45">
+        <f>IF(((T17*pax_cap*IF(B17="South Korea",korea_mid_load,load_mid)*IF(ABS(MOD(ABS((L17*M17*IF(B17="South Korea",korea_mid_revleg,revleg_mid))),1)-0.5)&lt;1E-9,2*ROUND((L17*M17*IF(B17="South Korea",korea_mid_revleg,revleg_mid))/2,0),ROUND((L17*M17*IF(B17="South Korea",korea_mid_revleg,revleg_mid)),0)))-(((battery/range_nm)*D17*IF(ABS(MOD(ABS((L17*M17*IF(B17="South Korea",korea_mid_revleg,revleg_mid))),1)-0.5)&lt;1E-9,2*ROUND((L17*M17*IF(B17="South Korea",korea_mid_revleg,revleg_mid))/2,0),ROUND((L17*M17*IF(B17="South Korea",korea_mid_revleg,revleg_mid)),0))*VLOOKUP(B17,country_opex,3,FALSE))+W17+X17+Y17+Z17+AA17))&lt;=0,"",VLOOKUP(B17,country_opex,7,FALSE)/((T17*pax_cap*IF(B17="South Korea",korea_mid_load,load_mid)*IF(ABS(MOD(ABS((L17*M17*IF(B17="South Korea",korea_mid_revleg,revleg_mid))),1)-0.5)&lt;1E-9,2*ROUND((L17*M17*IF(B17="South Korea",korea_mid_revleg,revleg_mid))/2,0),ROUND((L17*M17*IF(B17="South Korea",korea_mid_revleg,revleg_mid)),0)))-(((battery/range_nm)*D17*IF(ABS(MOD(ABS((L17*M17*IF(B17="South Korea",korea_mid_revleg,revleg_mid))),1)-0.5)&lt;1E-9,2*ROUND((L17*M17*IF(B17="South Korea",korea_mid_revleg,revleg_mid))/2,0),ROUND((L17*M17*IF(B17="South Korea",korea_mid_revleg,revleg_mid)),0))*VLOOKUP(B17,country_opex,3,FALSE))+W17+X17+Y17+Z17+AA17)))</f>
+        <v/>
+      </c>
+      <c r="AX17" s="45">
+        <f>IF(((T17*pax_cap*load_full*IF(ABS(MOD(ABS((L17*M17*revleg_full)),1)-0.5)&lt;1E-9,2*ROUND((L17*M17*revleg_full)/2,0),ROUND((L17*M17*revleg_full),0)))-(((battery/range_nm)*D17*IF(ABS(MOD(ABS((L17*M17*revleg_full)),1)-0.5)&lt;1E-9,2*ROUND((L17*M17*revleg_full)/2,0),ROUND((L17*M17*revleg_full),0))*VLOOKUP(B17,country_opex,3,FALSE))+W17+X17+Y17+Z17+AA17))&lt;=0,"",VLOOKUP(B17,country_opex,7,FALSE)/((T17*pax_cap*load_full*IF(ABS(MOD(ABS((L17*M17*revleg_full)),1)-0.5)&lt;1E-9,2*ROUND((L17*M17*revleg_full)/2,0),ROUND((L17*M17*revleg_full),0)))-(((battery/range_nm)*D17*IF(ABS(MOD(ABS((L17*M17*revleg_full)),1)-0.5)&lt;1E-9,2*ROUND((L17*M17*revleg_full)/2,0),ROUND((L17*M17*revleg_full),0))*VLOOKUP(B17,country_opex,3,FALSE))+W17+X17+Y17+Z17+AA17)))</f>
+        <v/>
+      </c>
+      <c r="AY17" s="46" t="inlineStr">
+        <is>
+          <t>https://www.yelapa.info/transport1.html</t>
+        </is>
+      </c>
+      <c r="AZ17" s="46" t="n"/>
+      <c r="BA17" s="34" t="inlineStr">
+        <is>
+          <t>ics-89a8844858</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="31" t="inlineStr">
+        <is>
+          <t>Mexico Pacific</t>
+        </is>
+      </c>
+      <c r="B18" s="31" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="C18" s="32" t="inlineStr">
+        <is>
+          <t>Cabo San Lucas Marina → Los Cabos, Baja Sur</t>
+        </is>
+      </c>
+      <c r="D18" s="33" t="n">
+        <v>17</v>
+      </c>
+      <c r="E18" s="27" t="n"/>
+      <c r="F18" s="34" t="n"/>
+      <c r="G18" s="34" t="n"/>
+      <c r="H18" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="I18" s="35">
+        <f>60*D18/cruise_kt</f>
+        <v/>
+      </c>
+      <c r="J18" s="35">
+        <f>IF(B18="South Korea",D18/korea_charge_range_nm*korea_full_range_charge_min,0)</f>
+        <v/>
+      </c>
+      <c r="K18" s="35">
+        <f>IF(B18="South Korea",I18+korea_turn_min+korea_dwell_min+J18,I18+turn_min+dwell_min)</f>
+        <v/>
+      </c>
+      <c r="L18" s="36">
+        <f>IF(B18="South Korea",FLOOR(60*korea_service_hr/K18,1),MIN(15,FLOOR(60*service_hr/K18,1)))</f>
+        <v/>
+      </c>
+      <c r="M18" s="36">
+        <f>IF(ABS(MOD(ABS((365*mech_uptime*H18)),1)-0.5)&lt;1E-9,2*ROUND((365*mech_uptime*H18)/2,0),ROUND((365*mech_uptime*H18),0))</f>
+        <v/>
+      </c>
+      <c r="N18" s="37">
+        <f>mech_uptime</f>
+        <v/>
+      </c>
+      <c r="O18" s="37">
+        <f>IF(AND(B18="South Korea",scenario="MID"),korea_mid_revleg,revleg_sel)</f>
+        <v/>
+      </c>
+      <c r="P18" s="36">
+        <f>IF(ABS(MOD(ABS((L18*M18*O18)),1)-0.5)&lt;1E-9,2*ROUND((L18*M18*O18)/2,0),ROUND((L18*M18*O18),0))</f>
+        <v/>
+      </c>
+      <c r="Q18" s="37">
+        <f>IF(AND(B18="South Korea",scenario="MID"),korea_mid_load,load_sel)</f>
+        <v/>
+      </c>
+      <c r="R18" s="38">
+        <f>pax_cap*Q18</f>
+        <v/>
+      </c>
+      <c r="S18" s="36">
+        <f>R18*P18</f>
+        <v/>
+      </c>
+      <c r="T18" s="39">
+        <f>E18*discount</f>
+        <v/>
+      </c>
+      <c r="U18" s="40">
+        <f>T18*S18</f>
+        <v/>
+      </c>
+      <c r="V18" s="40">
+        <f>(battery/range_nm)*D18*P18*VLOOKUP(B18,country_opex,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="W18" s="40">
+        <f>VLOOKUP(B18,country_opex,2,FALSE)*crew_factor</f>
+        <v/>
+      </c>
+      <c r="X18" s="40">
+        <f>VLOOKUP(B18,country_opex,5,FALSE)</f>
+        <v/>
+      </c>
+      <c r="Y18" s="40">
+        <f>maint</f>
+        <v/>
+      </c>
+      <c r="Z18" s="40">
+        <f>VLOOKUP(B18,country_opex,7,FALSE)*ins_pct</f>
+        <v/>
+      </c>
+      <c r="AA18" s="40">
+        <f>charge_berth</f>
+        <v/>
+      </c>
+      <c r="AB18" s="40">
+        <f>V18+W18+X18+Y18+Z18+AA18</f>
+        <v/>
+      </c>
+      <c r="AC18" s="40">
+        <f>VLOOKUP(B18,country_opex,7,FALSE)/dep_years</f>
+        <v/>
+      </c>
+      <c r="AD18" s="40">
+        <f>U18-AB18</f>
+        <v/>
+      </c>
+      <c r="AE18" s="37">
+        <f>IF(U18=0,"",AD18/U18)</f>
+        <v/>
+      </c>
+      <c r="AF18" s="38">
+        <f>IF(AD18&lt;=0,"",VLOOKUP(B18,country_opex,7,FALSE)/AD18)</f>
+        <v/>
+      </c>
+      <c r="AG18" s="35">
+        <f>((D18*P18/diesel_nmpg)*diesel_co2pg-(battery/range_nm)*D18*P18*VLOOKUP(B18,country_opex,4,FALSE))/1000</f>
+        <v/>
+      </c>
+      <c r="AH18" s="33" t="n"/>
+      <c r="AI18" s="34" t="n"/>
+      <c r="AJ18" s="34" t="n"/>
+      <c r="AK18" s="41" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="AL18" s="36">
+        <f>IF(AH18="","",AH18*AK18)</f>
+        <v/>
+      </c>
+      <c r="AM18" s="36">
+        <f>IF(OR(AH18="",S18=0),"",MIN(IF(AU18="",9.9E+99,AU18),FLOOR(AL18/S18,1)))</f>
+        <v/>
+      </c>
+      <c r="AN18" s="40">
+        <f>IF(AM18="","",AM18*IF(ABS(MOD(ABS((U18)),1)-0.5)&lt;1E-9,2*ROUND((U18)/2,0),ROUND((U18),0)))</f>
+        <v/>
+      </c>
+      <c r="AO18" s="38">
+        <f>IF(OR(AH18="",S18=0),"",MIN(IF(AU18="",9.9E+99,AU18),AL18/S18))</f>
+        <v/>
+      </c>
+      <c r="AP18" s="40">
+        <f>IF(AO18="","",AO18*IF(B18="South Korea",IF(ABS(MOD(ABS((U18)),1)-0.5)&lt;1E-9,2*ROUND((U18)/2,0),ROUND((U18),0)),U18))</f>
+        <v/>
+      </c>
+      <c r="AQ18" s="42" t="n"/>
+      <c r="AR18" s="34" t="inlineStr">
+        <is>
+          <t>Estimated</t>
+        </is>
+      </c>
+      <c r="AS18" s="43" t="n"/>
+      <c r="AT18" s="43" t="n"/>
+      <c r="AU18" s="44" t="n"/>
+      <c r="AV18" s="45">
+        <f>IF(((T18*pax_cap*load_thin*IF(ABS(MOD(ABS((L18*M18*revleg_thin)),1)-0.5)&lt;1E-9,2*ROUND((L18*M18*revleg_thin)/2,0),ROUND((L18*M18*revleg_thin),0)))-(((battery/range_nm)*D18*IF(ABS(MOD(ABS((L18*M18*revleg_thin)),1)-0.5)&lt;1E-9,2*ROUND((L18*M18*revleg_thin)/2,0),ROUND((L18*M18*revleg_thin),0))*VLOOKUP(B18,country_opex,3,FALSE))+W18+X18+Y18+Z18+AA18))&lt;=0,"",VLOOKUP(B18,country_opex,7,FALSE)/((T18*pax_cap*load_thin*IF(ABS(MOD(ABS((L18*M18*revleg_thin)),1)-0.5)&lt;1E-9,2*ROUND((L18*M18*revleg_thin)/2,0),ROUND((L18*M18*revleg_thin),0)))-(((battery/range_nm)*D18*IF(ABS(MOD(ABS((L18*M18*revleg_thin)),1)-0.5)&lt;1E-9,2*ROUND((L18*M18*revleg_thin)/2,0),ROUND((L18*M18*revleg_thin),0))*VLOOKUP(B18,country_opex,3,FALSE))+W18+X18+Y18+Z18+AA18)))</f>
+        <v/>
+      </c>
+      <c r="AW18" s="45">
+        <f>IF(((T18*pax_cap*IF(B18="South Korea",korea_mid_load,load_mid)*IF(ABS(MOD(ABS((L18*M18*IF(B18="South Korea",korea_mid_revleg,revleg_mid))),1)-0.5)&lt;1E-9,2*ROUND((L18*M18*IF(B18="South Korea",korea_mid_revleg,revleg_mid))/2,0),ROUND((L18*M18*IF(B18="South Korea",korea_mid_revleg,revleg_mid)),0)))-(((battery/range_nm)*D18*IF(ABS(MOD(ABS((L18*M18*IF(B18="South Korea",korea_mid_revleg,revleg_mid))),1)-0.5)&lt;1E-9,2*ROUND((L18*M18*IF(B18="South Korea",korea_mid_revleg,revleg_mid))/2,0),ROUND((L18*M18*IF(B18="South Korea",korea_mid_revleg,revleg_mid)),0))*VLOOKUP(B18,country_opex,3,FALSE))+W18+X18+Y18+Z18+AA18))&lt;=0,"",VLOOKUP(B18,country_opex,7,FALSE)/((T18*pax_cap*IF(B18="South Korea",korea_mid_load,load_mid)*IF(ABS(MOD(ABS((L18*M18*IF(B18="South Korea",korea_mid_revleg,revleg_mid))),1)-0.5)&lt;1E-9,2*ROUND((L18*M18*IF(B18="South Korea",korea_mid_revleg,revleg_mid))/2,0),ROUND((L18*M18*IF(B18="South Korea",korea_mid_revleg,revleg_mid)),0)))-(((battery/range_nm)*D18*IF(ABS(MOD(ABS((L18*M18*IF(B18="South Korea",korea_mid_revleg,revleg_mid))),1)-0.5)&lt;1E-9,2*ROUND((L18*M18*IF(B18="South Korea",korea_mid_revleg,revleg_mid))/2,0),ROUND((L18*M18*IF(B18="South Korea",korea_mid_revleg,revleg_mid)),0))*VLOOKUP(B18,country_opex,3,FALSE))+W18+X18+Y18+Z18+AA18)))</f>
+        <v/>
+      </c>
+      <c r="AX18" s="45">
+        <f>IF(((T18*pax_cap*load_full*IF(ABS(MOD(ABS((L18*M18*revleg_full)),1)-0.5)&lt;1E-9,2*ROUND((L18*M18*revleg_full)/2,0),ROUND((L18*M18*revleg_full),0)))-(((battery/range_nm)*D18*IF(ABS(MOD(ABS((L18*M18*revleg_full)),1)-0.5)&lt;1E-9,2*ROUND((L18*M18*revleg_full)/2,0),ROUND((L18*M18*revleg_full),0))*VLOOKUP(B18,country_opex,3,FALSE))+W18+X18+Y18+Z18+AA18))&lt;=0,"",VLOOKUP(B18,country_opex,7,FALSE)/((T18*pax_cap*load_full*IF(ABS(MOD(ABS((L18*M18*revleg_full)),1)-0.5)&lt;1E-9,2*ROUND((L18*M18*revleg_full)/2,0),ROUND((L18*M18*revleg_full),0)))-(((battery/range_nm)*D18*IF(ABS(MOD(ABS((L18*M18*revleg_full)),1)-0.5)&lt;1E-9,2*ROUND((L18*M18*revleg_full)/2,0),ROUND((L18*M18*revleg_full),0))*VLOOKUP(B18,country_opex,3,FALSE))+W18+X18+Y18+Z18+AA18)))</f>
+        <v/>
+      </c>
+      <c r="AY18" s="46" t="n"/>
+      <c r="AZ18" s="46" t="n"/>
+      <c r="BA18" s="34" t="inlineStr">
+        <is>
           <t>ics-db0930d9d1</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="47" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="47" t="inlineStr">
         <is>
           <t>TOTAL / median</t>
         </is>
       </c>
-      <c r="U16" s="48">
-        <f>SUM(U4:U15)</f>
-        <v/>
-      </c>
-      <c r="AD16" s="48">
-        <f>SUM(AD4:AD15)</f>
-        <v/>
-      </c>
-      <c r="AE16" s="49">
-        <f>IF(U16=0,"",AD16/U16)</f>
-        <v/>
-      </c>
-      <c r="AM16" s="50">
-        <f>SUM(AM4:AM15)</f>
-        <v/>
-      </c>
-      <c r="AN16" s="48">
-        <f>SUM(AN4:AN15)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="9" t="inlineStr">
+      <c r="U19" s="48">
+        <f>SUM(U4:U18)</f>
+        <v/>
+      </c>
+      <c r="AD19" s="48">
+        <f>SUM(AD4:AD18)</f>
+        <v/>
+      </c>
+      <c r="AE19" s="49">
+        <f>IF(U19=0,"",AD19/U19)</f>
+        <v/>
+      </c>
+      <c r="AM19" s="50">
+        <f>SUM(AM4:AM18)</f>
+        <v/>
+      </c>
+      <c r="AN19" s="48">
+        <f>SUM(AN4:AN18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="9" t="inlineStr">
         <is>
           <t>Market fleet build-up — grounded floor (network-sum of raw vessel fractions per market, rounded once; subset slices excluded; legacy per-corridor-floor totals above kept for reference)</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="25" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="25" t="inlineStr">
         <is>
           <t>Market</t>
         </is>
       </c>
-      <c r="B19" s="25" t="inlineStr">
+      <c r="B22" s="25" t="inlineStr">
         <is>
           <t>Fleet basis</t>
         </is>
       </c>
-      <c r="C19" s="25" t="inlineStr">
+      <c r="C22" s="25" t="inlineStr">
         <is>
           <t>Raw vessels (sum)</t>
         </is>
       </c>
-      <c r="D19" s="25" t="inlineStr">
+      <c r="D22" s="25" t="inlineStr">
         <is>
           <t>Fleet (rounded once)</t>
         </is>
       </c>
-      <c r="E19" s="25" t="inlineStr">
+      <c r="E22" s="25" t="inlineStr">
         <is>
           <t>Market rev/yr (raw sum)</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="26" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="26" t="inlineStr">
         <is>
           <t>Brazil</t>
         </is>
       </c>
-      <c r="B20" s="14" t="inlineStr">
+      <c r="B23" s="14" t="inlineStr">
         <is>
           <t>per_corridor_floor</t>
         </is>
       </c>
-      <c r="C20" s="14" t="inlineStr">
+      <c r="C23" s="14" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D20" s="51">
-        <f>SUMIFS(AM4:AM15,A4:A15,"Brazil",AQ4:AQ15,"=",AR4:AR15,"Grounded")</f>
-        <v/>
-      </c>
-      <c r="E20" s="52">
-        <f>SUMIFS(AN4:AN15,A4:A15,"Brazil",AQ4:AQ15,"=",AR4:AR15,"Grounded")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="26" t="inlineStr">
+      <c r="D23" s="51">
+        <f>SUMIFS(AM4:AM18,A4:A18,"Brazil",AQ4:AQ18,"=",AR4:AR18,"Grounded")</f>
+        <v/>
+      </c>
+      <c r="E23" s="52">
+        <f>SUMIFS(AN4:AN18,A4:A18,"Brazil",AQ4:AQ18,"=",AR4:AR18,"Grounded")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="26" t="inlineStr">
         <is>
           <t>Mexico Caribbean</t>
         </is>
       </c>
-      <c r="B21" s="14" t="inlineStr">
+      <c r="B24" s="14" t="inlineStr">
         <is>
           <t>grounded</t>
         </is>
       </c>
-      <c r="C21" s="14" t="inlineStr">
+      <c r="C24" s="14" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D21" s="51">
-        <f>SUMIFS(AM4:AM15,A4:A15,"Mexico Caribbean",AQ4:AQ15,"=",AR4:AR15,"Grounded")</f>
-        <v/>
-      </c>
-      <c r="E21" s="52">
-        <f>SUMIFS(AN4:AN15,A4:A15,"Mexico Caribbean",AQ4:AQ15,"=",AR4:AR15,"Grounded")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="26" t="inlineStr">
+      <c r="D24" s="51">
+        <f>SUMIFS(AM4:AM18,A4:A18,"Mexico Caribbean",AQ4:AQ18,"=",AR4:AR18,"Grounded")</f>
+        <v/>
+      </c>
+      <c r="E24" s="52">
+        <f>SUMIFS(AN4:AN18,A4:A18,"Mexico Caribbean",AQ4:AQ18,"=",AR4:AR18,"Grounded")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="26" t="inlineStr">
         <is>
           <t>Mexico Pacific</t>
         </is>
       </c>
-      <c r="B22" s="14" t="inlineStr">
+      <c r="B25" s="14" t="inlineStr">
         <is>
           <t>grounded</t>
         </is>
       </c>
-      <c r="C22" s="14" t="inlineStr">
+      <c r="C25" s="14" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D22" s="51">
-        <f>SUMIFS(AM4:AM15,A4:A15,"Mexico Pacific",AQ4:AQ15,"=",AR4:AR15,"Grounded")</f>
-        <v/>
-      </c>
-      <c r="E22" s="52">
-        <f>SUMIFS(AN4:AN15,A4:A15,"Mexico Pacific",AQ4:AQ15,"=",AR4:AR15,"Grounded")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="47" t="inlineStr">
+      <c r="D25" s="51">
+        <f>SUMIFS(AM4:AM18,A4:A18,"Mexico Pacific",AQ4:AQ18,"=",AR4:AR18,"Grounded")</f>
+        <v/>
+      </c>
+      <c r="E25" s="52">
+        <f>SUMIFS(AN4:AN18,A4:A18,"Mexico Pacific",AQ4:AQ18,"=",AR4:AR18,"Grounded")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="47" t="inlineStr">
         <is>
           <t>GROUNDED FLOOR (PUBLISHED)</t>
         </is>
       </c>
-      <c r="D23" s="50">
-        <f>SUM(D20:D22)</f>
-        <v/>
-      </c>
-      <c r="E23" s="48">
-        <f>SUM(E20:E22)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="21" t="inlineStr">
+      <c r="D26" s="50">
+        <f>SUM(D23:D25)</f>
+        <v/>
+      </c>
+      <c r="E26" s="48">
+        <f>SUM(E23:E25)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="21" t="inlineStr">
         <is>
           <t>ESTIMATED DEMAND (country-median cascade; held OUT of grounded floor)</t>
         </is>
       </c>
-      <c r="D24" s="53">
-        <f>SUMIF(AR4:AR15,"Estimated",AM4:AM15)</f>
-        <v/>
-      </c>
-      <c r="E24" s="54">
-        <f>SUMIF(AR4:AR15,"Estimated",AN4:AN15)</f>
+      <c r="D27" s="53">
+        <f>SUMIF(AR4:AR18,"Estimated",AM4:AM18)</f>
+        <v/>
+      </c>
+      <c r="E27" s="54">
+        <f>SUMIF(AR4:AR18,"Estimated",AN4:AN18)</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
+    <mergeCell ref="A21:L21"/>
     <mergeCell ref="A1:L1"/>
-    <mergeCell ref="A18:L18"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5435,7 +6035,7 @@
         </is>
       </c>
       <c r="C11" s="55">
-        <f>som_floor_rev/(ROUND(SUMPRODUCT(--('Corridor economics'!$AR$4:$AR$15="Grounded"),'Corridor economics'!$AH$4:$AH$15,'Corridor economics'!$E$4:$E$15),0))</f>
+        <f>som_floor_rev/(ROUND(SUMPRODUCT(--('Corridor economics'!$AR$4:$AR$18="Grounded"),'Corridor economics'!$AH$4:$AH$18,'Corridor economics'!$E$4:$E$18),0))</f>
         <v/>
       </c>
       <c r="E11" s="15" t="inlineStr">
@@ -5501,7 +6101,7 @@
         </is>
       </c>
       <c r="C16" s="52">
-        <f>ROUND(SUMPRODUCT(--('Corridor economics'!$AR$4:$AR$15="Grounded"),'Corridor economics'!$AH$4:$AH$15,'Corridor economics'!$E$4:$E$15),0)</f>
+        <f>ROUND(SUMPRODUCT(--('Corridor economics'!$AR$4:$AR$18="Grounded"),'Corridor economics'!$AH$4:$AH$18,'Corridor economics'!$E$4:$E$18),0)</f>
         <v/>
       </c>
       <c r="E16" s="15" t="inlineStr">

</xml_diff>

<commit_message>
Seal Angra/Floripa PROV corridors; re-apply Brazil+Egypt TAM decks
Grok handoff after #292:
- Seal rn-angra-abraao, rn-floripa-r3, rn-floripa-r4 geometry (land_km=0)
  into ROUTES/CLUSTERS/FEATURES; repoint finance + bindings pending→supported
- Regenerate DiDi/inDrive Brazil + Egypt deck economics (7-corridor floor)
- Live Slides re-apply: city marquees + 5/4-rung TAM ladders
- Refresh DiDi/inDrive/master transparent sheets (Drive in-place)

Sealed IDs: rn-7ec802385553, rn-36dcca92d821, rn-7d157e1300da
</commit_message>
<xml_diff>
--- a/finance/_refresh_didi.xlsx
+++ b/finance/_refresh_didi.xlsx
@@ -3156,11 +3156,11 @@
       </c>
       <c r="C6" s="32" t="inlineStr">
         <is>
-          <t>Beira Mar Terminal (continent) → Miramar Terminal (Florianopolis island)</t>
+          <t>Barreiros Terminal (Sao Jose / continent) → Miramar Terminal (Florianopolis island)</t>
         </is>
       </c>
       <c r="D6" s="33" t="n">
-        <v>4.79</v>
+        <v>4.77</v>
       </c>
       <c r="E6" s="27" t="n">
         <v>20</v>
@@ -3271,7 +3271,7 @@
         <v/>
       </c>
       <c r="AH6" s="33" t="n">
-        <v>6100556</v>
+        <v>3890964</v>
       </c>
       <c r="AI6" s="34" t="inlineStr">
         <is>
@@ -3335,7 +3335,7 @@
       </c>
       <c r="BA6" s="34" t="inlineStr">
         <is>
-          <t>rn-floripa-r4-PROV</t>
+          <t>rn-36dcca92d821</t>
         </is>
       </c>
     </row>
@@ -3352,11 +3352,11 @@
       </c>
       <c r="C7" s="32" t="inlineStr">
         <is>
-          <t>Barreiros Terminal (Sao Jose / continent) → Miramar Terminal (Florianopolis island)</t>
+          <t>Beira Mar Terminal (continent) → Miramar Terminal (Florianopolis island)</t>
         </is>
       </c>
       <c r="D7" s="33" t="n">
-        <v>4.99</v>
+        <v>5.15</v>
       </c>
       <c r="E7" s="27" t="n">
         <v>20</v>
@@ -3467,7 +3467,7 @@
         <v/>
       </c>
       <c r="AH7" s="33" t="n">
-        <v>3890964</v>
+        <v>6100556</v>
       </c>
       <c r="AI7" s="34" t="inlineStr">
         <is>
@@ -3531,7 +3531,7 @@
       </c>
       <c r="BA7" s="34" t="inlineStr">
         <is>
-          <t>rn-floripa-r3-PROV</t>
+          <t>rn-7d157e1300da</t>
         </is>
       </c>
     </row>
@@ -4155,7 +4155,7 @@
       </c>
       <c r="BA10" s="34" t="inlineStr">
         <is>
-          <t>rn-angra-abraao-PROV</t>
+          <t>rn-7ec802385553</t>
         </is>
       </c>
     </row>

</xml_diff>